<commit_message>
Correct flux processing and align tree-surface scaling
</commit_message>
<xml_diff>
--- a/data processing/goFlux_reprocessing/ymf_black_oak/results/CH4_best_YMF.xlsx
+++ b/data processing/goFlux_reprocessing/ymf_black_oak/results/CH4_best_YMF.xlsx
@@ -146,10 +146,10 @@
     <t xml:space="preserve">YMF_0.5m</t>
   </si>
   <si>
-    <t xml:space="preserve">MDF (HM)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MDF (LM)</t>
+    <t xml:space="preserve">Noise (HM.MAE) | MDF (HM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Noise (LM.MAE) | MDF (LM)</t>
   </si>
   <si>
     <t xml:space="preserve">HM</t>
@@ -161,24 +161,30 @@
     <t xml:space="preserve">YMF_1.25m</t>
   </si>
   <si>
+    <t xml:space="preserve">Noise (HM.MAE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Noise (LM.MAE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AICc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YMF_10m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YMF_2m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YMF_4m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YMF_4m_restart</t>
+  </si>
+  <si>
     <t xml:space="preserve"/>
   </si>
   <si>
-    <t xml:space="preserve">AICc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">YMF_10m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">YMF_2m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">YMF_4m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">YMF_4m_restart</t>
-  </si>
-  <si>
     <t xml:space="preserve">YMF_6m</t>
   </si>
   <si>
@@ -186,12 +192,6 @@
   </si>
   <si>
     <t xml:space="preserve">YMF_Seam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Noise (HM.MAE)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Noise (LM.MAE)</t>
   </si>
 </sst>
 </file>
@@ -656,7 +656,7 @@
         <v>43</v>
       </c>
       <c r="B2" t="n">
-        <v>-0.00396562808995602</v>
+        <v>-0.00389395255460912</v>
       </c>
       <c r="C2" t="n">
         <v>1940.80910604831</v>
@@ -677,10 +677,10 @@
         <v>191.382828544352</v>
       </c>
       <c r="I2" t="n">
-        <v>0.00812692966743516</v>
+        <v>0.00798004183087438</v>
       </c>
       <c r="J2" t="n">
-        <v>-204.934236975442</v>
+        <v>-204.934233762779</v>
       </c>
       <c r="K2" t="n">
         <v>-0.016477614613488</v>
@@ -689,37 +689,37 @@
         <v>0.627895065283225</v>
       </c>
       <c r="M2" t="n">
-        <v>-0.00476396815325628</v>
+        <v>-0.00514805392791875</v>
       </c>
       <c r="N2" t="n">
-        <v>1940.82782316954</v>
+        <v>1940.83799528314</v>
       </c>
       <c r="O2" t="n">
-        <v>1939.14598229509</v>
+        <v>1939.64813781309</v>
       </c>
       <c r="P2" t="n">
-        <v>-0.00208128775907568</v>
+        <v>-0.00229048627945938</v>
       </c>
       <c r="Q2" t="n">
-        <v>1.32886411691635</v>
+        <v>1.32884086414351</v>
       </c>
       <c r="R2" t="n">
-        <v>1.6590185751789</v>
+        <v>1.65883296432331</v>
       </c>
       <c r="S2" t="n">
-        <v>193.746047690497</v>
+        <v>193.735306617882</v>
       </c>
       <c r="T2" t="n">
-        <v>0.0358462690810641</v>
+        <v>0.0372661432018119</v>
       </c>
       <c r="U2" t="n">
-        <v>-752.445606853235</v>
+        <v>-723.887972496003</v>
       </c>
       <c r="V2" t="n">
-        <v>-0.0160211732658191</v>
+        <v>-0.0157938412604248</v>
       </c>
       <c r="W2" t="n">
-        <v>0.00123750575378016</v>
+        <v>0.00192500895032469</v>
       </c>
       <c r="X2" t="n">
         <v>1940.47</v>
@@ -728,25 +728,25 @@
         <v>1940.83</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.0136363108593246</v>
+        <v>0.00860775783296085</v>
       </c>
       <c r="AA2" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="AB2" t="n">
-        <v>2.28895217995805</v>
+        <v>2.24758121193978</v>
       </c>
       <c r="AC2" t="n">
         <v>48</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.00123750575378016</v>
+        <v>0.00192500895032469</v>
       </c>
       <c r="AE2" t="n">
         <v>1</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.20131491032209</v>
+        <v>1.32206385561252</v>
       </c>
       <c r="AG2" t="s">
         <v>44</v>
@@ -755,7 +755,7 @@
         <v>45</v>
       </c>
       <c r="AI2" t="n">
-        <v>-0.00476396815325628</v>
+        <v>-0.00514805392791875</v>
       </c>
       <c r="AJ2" t="s">
         <v>46</v>
@@ -770,7 +770,7 @@
         <v>1</v>
       </c>
       <c r="AN2" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="AO2" t="n">
         <v>2</v>
@@ -779,7 +779,7 @@
         <v>0.5</v>
       </c>
       <c r="AQ2" t="n">
-        <v>0.014</v>
+        <v>0.0086</v>
       </c>
     </row>
     <row r="3">
@@ -787,7 +787,7 @@
         <v>48</v>
       </c>
       <c r="B3" t="n">
-        <v>0.0380952811319747</v>
+        <v>0.037406739592681</v>
       </c>
       <c r="C3" t="n">
         <v>1937.40836522261</v>
@@ -808,10 +808,10 @@
         <v>254.20018976306</v>
       </c>
       <c r="I3" t="n">
-        <v>0.002895434516631</v>
+        <v>0.00284310155799923</v>
       </c>
       <c r="J3" t="n">
-        <v>7.60050701975461</v>
+        <v>7.60050618941276</v>
       </c>
       <c r="K3" t="n">
         <v>0.693680686527493</v>
@@ -820,7 +820,7 @@
         <v>0.00000000000000000000358541741421322</v>
       </c>
       <c r="M3" t="n">
-        <v>0.0452083702163778</v>
+        <v>0.0443912653180071</v>
       </c>
       <c r="N3" t="n">
         <v>1937.22162373941</v>
@@ -841,10 +841,10 @@
         <v>256.029255781137</v>
       </c>
       <c r="T3" t="n">
-        <v>0.0130702897306643</v>
+        <v>0.0128340533634279</v>
       </c>
       <c r="U3" t="n">
-        <v>28.9112163701255</v>
+        <v>28.9112132116266</v>
       </c>
       <c r="V3" t="n">
         <v>0.695258815852541</v>
@@ -859,19 +859,19 @@
         <v>1942.4</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.00845621018302839</v>
+        <v>0.00533788135156456</v>
       </c>
       <c r="AA3" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="AB3" t="n">
-        <v>2.2892168995484</v>
+        <v>2.24784114693663</v>
       </c>
       <c r="AC3" t="n">
         <v>77</v>
       </c>
       <c r="AD3" t="n">
-        <v>0.0118865604651248</v>
+        <v>0.018490205167972</v>
       </c>
       <c r="AE3" t="n">
         <v>1</v>
@@ -883,16 +883,16 @@
         <v>49</v>
       </c>
       <c r="AH3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AI3" t="n">
-        <v>0.0452083702163778</v>
+        <v>0.0443912653180071</v>
       </c>
       <c r="AJ3" t="s">
         <v>46</v>
       </c>
       <c r="AK3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL3" t="n">
         <v>1</v>
@@ -901,7 +901,7 @@
         <v>1</v>
       </c>
       <c r="AN3" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="AO3" t="n">
         <v>2</v>
@@ -910,15 +910,15 @@
         <v>0.5</v>
       </c>
       <c r="AQ3" t="n">
-        <v>0.0085</v>
+        <v>0.0053</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B4" t="n">
-        <v>0.0267625203970198</v>
+        <v>0.0265423992919272</v>
       </c>
       <c r="C4" t="n">
         <v>1943.57896641938</v>
@@ -939,10 +939,10 @@
         <v>597.623661463038</v>
       </c>
       <c r="I4" t="n">
-        <v>0.00155846889284365</v>
+        <v>0.00154565025168617</v>
       </c>
       <c r="J4" t="n">
-        <v>5.82332631502523</v>
+        <v>5.82332529431986</v>
       </c>
       <c r="K4" t="n">
         <v>0.665073921237439</v>
@@ -951,7 +951,7 @@
         <v>0.000000000000000000000000000000000000590562629747041</v>
       </c>
       <c r="M4" t="n">
-        <v>0.0309385078107122</v>
+        <v>0.0306840393066931</v>
       </c>
       <c r="N4" t="n">
         <v>1943.3638234807</v>
@@ -972,10 +972,10 @@
         <v>599.354005809485</v>
       </c>
       <c r="T4" t="n">
-        <v>0.00692457399247662</v>
+        <v>0.00686761832939888</v>
       </c>
       <c r="U4" t="n">
-        <v>22.3817322892316</v>
+        <v>22.3817283661896</v>
       </c>
       <c r="V4" t="n">
         <v>0.665931303103025</v>
@@ -990,19 +990,19 @@
         <v>1953.57</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.00435962955646659</v>
+        <v>0.00277956752477507</v>
       </c>
       <c r="AA4" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="AB4" t="n">
-        <v>2.29503355936848</v>
+        <v>2.2761569619547</v>
       </c>
       <c r="AC4" t="n">
         <v>149</v>
       </c>
       <c r="AD4" t="n">
-        <v>0.00832932743830177</v>
+        <v>0.0129567315706916</v>
       </c>
       <c r="AE4" t="n">
         <v>1</v>
@@ -1014,16 +1014,16 @@
         <v>49</v>
       </c>
       <c r="AH4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AI4" t="n">
-        <v>0.0309385078107122</v>
+        <v>0.0306840393066931</v>
       </c>
       <c r="AJ4" t="s">
         <v>46</v>
       </c>
       <c r="AK4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL4" t="n">
         <v>1</v>
@@ -1032,7 +1032,7 @@
         <v>1</v>
       </c>
       <c r="AN4" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="AO4" t="n">
         <v>2</v>
@@ -1041,15 +1041,15 @@
         <v>0.5</v>
       </c>
       <c r="AQ4" t="n">
-        <v>0.0044</v>
+        <v>0.0028</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B5" t="n">
-        <v>0.0377476994393041</v>
+        <v>0.0371043179696165</v>
       </c>
       <c r="C5" t="n">
         <v>1934.80539572394</v>
@@ -1070,10 +1070,10 @@
         <v>268.461127892914</v>
       </c>
       <c r="I5" t="n">
-        <v>0.00457003841931834</v>
+        <v>0.0044921451703506</v>
       </c>
       <c r="J5" t="n">
-        <v>12.1067998505887</v>
+        <v>12.1067989284403</v>
       </c>
       <c r="K5" t="n">
         <v>0.497133148131768</v>
@@ -1082,7 +1082,7 @@
         <v>0.00000000000818447996951748</v>
       </c>
       <c r="M5" t="n">
-        <v>0.0377788214969031</v>
+        <v>0.0371349095748844</v>
       </c>
       <c r="N5" t="n">
         <v>1934.8042863122</v>
@@ -1103,10 +1103,10 @@
         <v>270.738816267576</v>
       </c>
       <c r="T5" t="n">
-        <v>0.0182541192865066</v>
+        <v>0.017942990029262</v>
       </c>
       <c r="U5" t="n">
-        <v>48.3183925893585</v>
+        <v>48.3183889086333</v>
       </c>
       <c r="V5" t="n">
         <v>0.496975719496566</v>
@@ -1121,19 +1121,19 @@
         <v>1940.05</v>
       </c>
       <c r="Z5" t="n">
-        <v>0.00946339990245041</v>
+        <v>0.00597992354203657</v>
       </c>
       <c r="AA5" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="AB5" t="n">
-        <v>2.29149469066478</v>
+        <v>2.25243786750044</v>
       </c>
       <c r="AC5" t="n">
         <v>69</v>
       </c>
       <c r="AD5" t="n">
-        <v>0.0117663997069196</v>
+        <v>0.018303288432986</v>
       </c>
       <c r="AE5" t="n">
         <v>1</v>
@@ -1145,16 +1145,16 @@
         <v>49</v>
       </c>
       <c r="AH5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AI5" t="n">
-        <v>0.0377788214969031</v>
+        <v>0.0371349095748844</v>
       </c>
       <c r="AJ5" t="s">
         <v>46</v>
       </c>
       <c r="AK5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL5" t="n">
         <v>1</v>
@@ -1163,7 +1163,7 @@
         <v>1</v>
       </c>
       <c r="AN5" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="AO5" t="n">
         <v>2</v>
@@ -1172,15 +1172,15 @@
         <v>0.5</v>
       </c>
       <c r="AQ5" t="n">
-        <v>0.0095</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B6" t="n">
-        <v>0.324616519777869</v>
+        <v>0.320860486165164</v>
       </c>
       <c r="C6" t="n">
         <v>1967.46703869648</v>
@@ -1201,10 +1201,10 @@
         <v>210.144435692446</v>
       </c>
       <c r="I6" t="n">
-        <v>0.00416110305989188</v>
+        <v>0.00411295551933168</v>
       </c>
       <c r="J6" t="n">
-        <v>1.28185191029072</v>
+        <v>1.28185167593822</v>
       </c>
       <c r="K6" t="n">
         <v>0.99007467292149</v>
@@ -1213,7 +1213,7 @@
         <v>0.0000000000000000000000000000000000000000000000000000000000000501306748403574</v>
       </c>
       <c r="M6" t="n">
-        <v>0.347487029392391</v>
+        <v>0.343466368449842</v>
       </c>
       <c r="N6" t="n">
         <v>1966.9817108955</v>
@@ -1234,10 +1234,10 @@
         <v>210.315714773105</v>
       </c>
       <c r="T6" t="n">
-        <v>0.0170503405639689</v>
+        <v>0.0168530534619548</v>
       </c>
       <c r="U6" t="n">
-        <v>4.90675597123231</v>
+        <v>4.90675507416264</v>
       </c>
       <c r="V6" t="n">
         <v>0.990407805013714</v>
@@ -1252,19 +1252,19 @@
         <v>2010</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.0105602732564386</v>
+        <v>0.00671019667865075</v>
       </c>
       <c r="AA6" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="AB6" t="n">
-        <v>2.29308790711238</v>
+        <v>2.26655532256648</v>
       </c>
       <c r="AC6" t="n">
         <v>62</v>
       </c>
       <c r="AD6" t="n">
-        <v>0.101116464824266</v>
+        <v>0.157292278615525</v>
       </c>
       <c r="AE6" t="n">
         <v>1</v>
@@ -1276,16 +1276,16 @@
         <v>49</v>
       </c>
       <c r="AH6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AI6" t="n">
-        <v>0.347487029392391</v>
+        <v>0.343466368449842</v>
       </c>
       <c r="AJ6" t="s">
         <v>46</v>
       </c>
       <c r="AK6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL6" t="n">
         <v>1</v>
@@ -1294,7 +1294,7 @@
         <v>1</v>
       </c>
       <c r="AN6" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="AO6" t="n">
         <v>2</v>
@@ -1303,15 +1303,15 @@
         <v>0.5</v>
       </c>
       <c r="AQ6" t="n">
-        <v>0.011</v>
+        <v>0.0067</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B7" t="n">
-        <v>0.36323187849675</v>
+        <v>0.358270947361978</v>
       </c>
       <c r="C7" t="n">
         <v>1966.14972056748</v>
@@ -1332,10 +1332,10 @@
         <v>390.37109254052</v>
       </c>
       <c r="I7" t="n">
-        <v>0.00159045054400966</v>
+        <v>0.00156872834189404</v>
       </c>
       <c r="J7" t="n">
-        <v>0.437860947280236</v>
+        <v>0.437860885300609</v>
       </c>
       <c r="K7" t="n">
         <v>0.997780915269485</v>
@@ -1344,7 +1344,7 @@
         <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000114790757577001</v>
       </c>
       <c r="M7" t="n">
-        <v>0.389685801481711</v>
+        <v>0.384363569211378</v>
       </c>
       <c r="N7" t="n">
         <v>1965.06581638193</v>
@@ -1365,10 +1365,10 @@
         <v>372.955730529914</v>
       </c>
       <c r="T7" t="n">
-        <v>0.00614558319564546</v>
+        <v>0.00606164748271379</v>
       </c>
       <c r="U7" t="n">
-        <v>1.57706110211816</v>
+        <v>1.57706087888372</v>
       </c>
       <c r="V7" t="n">
         <v>0.998122550225431</v>
@@ -1383,19 +1383,19 @@
         <v>2055.53</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.00555228585184914</v>
+        <v>0.00352057763911637</v>
       </c>
       <c r="AA7" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="AB7" t="n">
-        <v>2.29230087312057</v>
+        <v>2.26099319489918</v>
       </c>
       <c r="AC7" t="n">
         <v>117</v>
       </c>
       <c r="AD7" t="n">
-        <v>0.113183807948472</v>
+        <v>0.176063701253178</v>
       </c>
       <c r="AE7" t="n">
         <v>1</v>
@@ -1404,19 +1404,19 @@
         <v>1.07282929872356</v>
       </c>
       <c r="AG7" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="AH7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AI7" t="n">
-        <v>0.389685801481711</v>
+        <v>0.384363569211378</v>
       </c>
       <c r="AJ7" t="s">
         <v>46</v>
       </c>
       <c r="AK7" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="AL7" t="n">
         <v>0</v>
@@ -1425,7 +1425,7 @@
         <v>2</v>
       </c>
       <c r="AN7" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="AO7" t="n">
         <v>2</v>
@@ -1434,15 +1434,15 @@
         <v>0.5</v>
       </c>
       <c r="AQ7" t="n">
-        <v>0.0056</v>
+        <v>0.0035</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B8" t="n">
-        <v>0.0330522557112562</v>
+        <v>0.0326813688912162</v>
       </c>
       <c r="C8" t="n">
         <v>1947.05438749854</v>
@@ -1463,10 +1463,10 @@
         <v>584.769887790663</v>
       </c>
       <c r="I8" t="n">
-        <v>0.00103884901742328</v>
+        <v>0.00102719188740148</v>
       </c>
       <c r="J8" t="n">
-        <v>3.14305028527746</v>
+        <v>3.1430503747276</v>
       </c>
       <c r="K8" t="n">
         <v>0.859726359528916</v>
@@ -1475,7 +1475,7 @@
         <v>0.00000000000000000000000000000000000000000000000000000000000000000000000458762835603426</v>
       </c>
       <c r="M8" t="n">
-        <v>0.0331211007475123</v>
+        <v>0.0327494414017846</v>
       </c>
       <c r="N8" t="n">
         <v>1947.04959314447</v>
@@ -1496,10 +1496,10 @@
         <v>587.150515299484</v>
       </c>
       <c r="T8" t="n">
-        <v>0.00416021133861464</v>
+        <v>0.00411352878541541</v>
       </c>
       <c r="U8" t="n">
-        <v>12.5606071196988</v>
+        <v>12.5606074770828</v>
       </c>
       <c r="V8" t="n">
         <v>0.859492457974167</v>
@@ -1514,19 +1514,19 @@
         <v>1959.58</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.00390577680241217</v>
+        <v>0.00248268162826229</v>
       </c>
       <c r="AA8" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="AB8" t="n">
-        <v>2.29324895113058</v>
+        <v>2.26751588714622</v>
       </c>
       <c r="AC8" t="n">
         <v>166</v>
       </c>
       <c r="AD8" t="n">
-        <v>0.0102948936563689</v>
+        <v>0.0160142790210182</v>
       </c>
       <c r="AE8" t="n">
         <v>1</v>
@@ -1538,16 +1538,16 @@
         <v>49</v>
       </c>
       <c r="AH8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AI8" t="n">
-        <v>0.0331211007475123</v>
+        <v>0.0327494414017846</v>
       </c>
       <c r="AJ8" t="s">
         <v>46</v>
       </c>
       <c r="AK8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL8" t="n">
         <v>1</v>
@@ -1556,7 +1556,7 @@
         <v>1</v>
       </c>
       <c r="AN8" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="AO8" t="n">
         <v>2</v>
@@ -1565,15 +1565,15 @@
         <v>0.5</v>
       </c>
       <c r="AQ8" t="n">
-        <v>0.0039</v>
+        <v>0.0025</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B9" t="n">
-        <v>0.0747621536813002</v>
+        <v>0.0739757902704793</v>
       </c>
       <c r="C9" t="n">
         <v>1942.01519797732</v>
@@ -1594,10 +1594,10 @@
         <v>720.787312154195</v>
       </c>
       <c r="I9" t="n">
-        <v>0.000939850733863672</v>
+        <v>0.000929965167568801</v>
       </c>
       <c r="J9" t="n">
-        <v>1.25712099984454</v>
+        <v>1.25712096372144</v>
       </c>
       <c r="K9" t="n">
         <v>0.970695174412968</v>
@@ -1606,7 +1606,7 @@
         <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000814683212799519</v>
       </c>
       <c r="M9" t="n">
-        <v>0.0752279383883071</v>
+        <v>0.0744366757599961</v>
       </c>
       <c r="N9" t="n">
         <v>1941.98429200858</v>
@@ -1627,10 +1627,10 @@
         <v>723.967541406523</v>
       </c>
       <c r="T9" t="n">
-        <v>0.00377576832638016</v>
+        <v>0.00373605392625383</v>
       </c>
       <c r="U9" t="n">
-        <v>5.01910381604587</v>
+        <v>5.01910367182419</v>
       </c>
       <c r="V9" t="n">
         <v>0.97052787072339</v>
@@ -1645,19 +1645,19 @@
         <v>1975.14</v>
       </c>
       <c r="Z9" t="n">
-        <v>0.00338233849982336</v>
+        <v>0.00215149010227422</v>
       </c>
       <c r="AA9" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="AB9" t="n">
-        <v>2.29515826773728</v>
+        <v>2.27101733017835</v>
       </c>
       <c r="AC9" t="n">
         <v>192</v>
       </c>
       <c r="AD9" t="n">
-        <v>0.0232670396174607</v>
+        <v>0.0361931727382722</v>
       </c>
       <c r="AE9" t="n">
         <v>1</v>
@@ -1669,16 +1669,16 @@
         <v>49</v>
       </c>
       <c r="AH9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AI9" t="n">
-        <v>0.0752279383883071</v>
+        <v>0.0744366757599961</v>
       </c>
       <c r="AJ9" t="s">
         <v>46</v>
       </c>
       <c r="AK9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL9" t="n">
         <v>1</v>
@@ -1687,7 +1687,7 @@
         <v>1</v>
       </c>
       <c r="AN9" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="AO9" t="n">
         <v>2</v>
@@ -1696,15 +1696,15 @@
         <v>0.5</v>
       </c>
       <c r="AQ9" t="n">
-        <v>0.0034</v>
+        <v>0.0022</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B10" t="n">
-        <v>0.00949384276810327</v>
+        <v>0.00933809045098793</v>
       </c>
       <c r="C10" t="n">
         <v>1945.24081742601</v>
@@ -1725,10 +1725,10 @@
         <v>391.616128634832</v>
       </c>
       <c r="I10" t="n">
-        <v>0.00533051182276102</v>
+        <v>0.00524306284899662</v>
       </c>
       <c r="J10" t="n">
-        <v>56.1470413294613</v>
+        <v>56.1470557231744</v>
       </c>
       <c r="K10" t="n">
         <v>0.030518900730106</v>
@@ -1737,7 +1737,7 @@
         <v>0.0793724420639434</v>
       </c>
       <c r="M10" t="n">
-        <v>0.00948658459318646</v>
+        <v>0.00933095135088507</v>
       </c>
       <c r="N10" t="n">
         <v>1945.24116912113</v>
@@ -1758,10 +1758,10 @@
         <v>393.869122593964</v>
       </c>
       <c r="T10" t="n">
-        <v>0.025857210272933</v>
+        <v>0.0254330133882531</v>
       </c>
       <c r="U10" t="n">
-        <v>272.566064413787</v>
+        <v>272.566134275694</v>
       </c>
       <c r="V10" t="n">
         <v>0.0305018423219471</v>
@@ -1776,19 +1776,19 @@
         <v>1948.32</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.00560136934722782</v>
+        <v>0.00354180564350198</v>
       </c>
       <c r="AA10" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="AB10" t="n">
-        <v>2.28455849804792</v>
+        <v>2.24707891382181</v>
       </c>
       <c r="AC10" t="n">
         <v>70</v>
       </c>
       <c r="AD10" t="n">
-        <v>0.0029683268205762</v>
+        <v>0.00461739727645186</v>
       </c>
       <c r="AE10" t="n">
         <v>1</v>
@@ -1797,19 +1797,19 @@
         <v>0.999235486083549</v>
       </c>
       <c r="AG10" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="AH10" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="AI10" t="n">
-        <v>0.00948658459318646</v>
+        <v>0.00933095135088507</v>
       </c>
       <c r="AJ10" t="s">
         <v>46</v>
       </c>
       <c r="AK10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL10" t="n">
         <v>1</v>
@@ -1818,7 +1818,7 @@
         <v>1</v>
       </c>
       <c r="AN10" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="AO10" t="n">
         <v>2</v>
@@ -1827,7 +1827,7 @@
         <v>0.5</v>
       </c>
       <c r="AQ10" t="n">
-        <v>0.0056</v>
+        <v>0.0035</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Align empirical noise thresholds across flux fitting and detection
Estimate noise within closures and group by analyzer, day and logging interval. Use consistent physical durations for the pinned goFlux fits and reported MDFs, retain signed observations, and export precision diagnostics. Regenerate analyses and figures, add swamp component-budget scenarios and rate-area summaries, and document the independent workflow with regression checks.
</commit_message>
<xml_diff>
--- a/data processing/goFlux_reprocessing/ymf_black_oak/results/CH4_best_YMF.xlsx
+++ b/data processing/goFlux_reprocessing/ymf_black_oak/results/CH4_best_YMF.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
   <si>
     <t xml:space="preserve">UniqueID</t>
   </si>
@@ -146,10 +146,10 @@
     <t xml:space="preserve">YMF_0.5m</t>
   </si>
   <si>
-    <t xml:space="preserve">Noise (HM.MAE) | MDF (HM)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Noise (LM.MAE) | MDF (LM)</t>
+    <t xml:space="preserve">MDF (HM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MDF (LM)</t>
   </si>
   <si>
     <t xml:space="preserve">HM</t>
@@ -161,10 +161,7 @@
     <t xml:space="preserve">YMF_1.25m</t>
   </si>
   <si>
-    <t xml:space="preserve">Noise (HM.MAE)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Noise (LM.MAE)</t>
+    <t xml:space="preserve"/>
   </si>
   <si>
     <t xml:space="preserve">AICc</t>
@@ -180,9 +177,6 @@
   </si>
   <si>
     <t xml:space="preserve">YMF_4m_restart</t>
-  </si>
-  <si>
-    <t xml:space="preserve"/>
   </si>
   <si>
     <t xml:space="preserve">YMF_6m</t>
@@ -689,37 +683,37 @@
         <v>0.627895065283225</v>
       </c>
       <c r="M2" t="n">
-        <v>-0.00514805392791875</v>
+        <v>-0.00437387748466349</v>
       </c>
       <c r="N2" t="n">
-        <v>1940.83799528314</v>
+        <v>1940.82084652088</v>
       </c>
       <c r="O2" t="n">
-        <v>1939.64813781309</v>
+        <v>1938.3023913532</v>
       </c>
       <c r="P2" t="n">
-        <v>-0.00229048627945938</v>
+        <v>-0.00194603757204778</v>
       </c>
       <c r="Q2" t="n">
-        <v>1.32884086414351</v>
+        <v>1.32887634752365</v>
       </c>
       <c r="R2" t="n">
-        <v>1.65883296432331</v>
+        <v>1.65915297218831</v>
       </c>
       <c r="S2" t="n">
-        <v>193.735306617882</v>
+        <v>193.753824330568</v>
       </c>
       <c r="T2" t="n">
-        <v>0.0372661432018119</v>
+        <v>0.0338390513753052</v>
       </c>
       <c r="U2" t="n">
-        <v>-723.887972496003</v>
+        <v>-773.662533849154</v>
       </c>
       <c r="V2" t="n">
-        <v>-0.0157938412604248</v>
+        <v>-0.0161857955795053</v>
       </c>
       <c r="W2" t="n">
-        <v>0.00192500895032469</v>
+        <v>0.000772710825677044</v>
       </c>
       <c r="X2" t="n">
         <v>1940.47</v>
@@ -728,10 +722,10 @@
         <v>1940.83</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.00860775783296085</v>
+        <v>0.0210851045068941</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.9</v>
+        <v>2.2421169701799</v>
       </c>
       <c r="AB2" t="n">
         <v>2.24758121193978</v>
@@ -740,13 +734,13 @@
         <v>48</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.00192500895032469</v>
+        <v>0.000772710825677044</v>
       </c>
       <c r="AE2" t="n">
         <v>1</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.32206385561252</v>
+        <v>1.12324878727305</v>
       </c>
       <c r="AG2" t="s">
         <v>44</v>
@@ -755,7 +749,7 @@
         <v>45</v>
       </c>
       <c r="AI2" t="n">
-        <v>-0.00514805392791875</v>
+        <v>-0.00437387748466349</v>
       </c>
       <c r="AJ2" t="s">
         <v>46</v>
@@ -770,7 +764,7 @@
         <v>1</v>
       </c>
       <c r="AN2" t="n">
-        <v>0.9</v>
+        <v>2.2421169701799</v>
       </c>
       <c r="AO2" t="n">
         <v>2</v>
@@ -779,7 +773,7 @@
         <v>0.5</v>
       </c>
       <c r="AQ2" t="n">
-        <v>0.0086</v>
+        <v>0.021</v>
       </c>
     </row>
     <row r="3">
@@ -859,10 +853,10 @@
         <v>1942.4</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.00533788135156456</v>
+        <v>0.0131590673154446</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.9</v>
+        <v>2.2421169701799</v>
       </c>
       <c r="AB3" t="n">
         <v>2.24784114693663</v>
@@ -871,7 +865,7 @@
         <v>77</v>
       </c>
       <c r="AD3" t="n">
-        <v>0.018490205167972</v>
+        <v>0.00742208585569002</v>
       </c>
       <c r="AE3" t="n">
         <v>1</v>
@@ -883,7 +877,7 @@
         <v>49</v>
       </c>
       <c r="AH3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="AI3" t="n">
         <v>0.0443912653180071</v>
@@ -892,7 +886,7 @@
         <v>46</v>
       </c>
       <c r="AK3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="AL3" t="n">
         <v>1</v>
@@ -901,7 +895,7 @@
         <v>1</v>
       </c>
       <c r="AN3" t="n">
-        <v>0.9</v>
+        <v>2.2421169701799</v>
       </c>
       <c r="AO3" t="n">
         <v>2</v>
@@ -910,12 +904,12 @@
         <v>0.5</v>
       </c>
       <c r="AQ3" t="n">
-        <v>0.0053</v>
+        <v>0.013</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B4" t="n">
         <v>0.0265423992919272</v>
@@ -990,10 +984,10 @@
         <v>1953.57</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.00277956752477507</v>
+        <v>0.00688719318649359</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.9</v>
+        <v>2.2421169701799</v>
       </c>
       <c r="AB4" t="n">
         <v>2.2761569619547</v>
@@ -1002,7 +996,7 @@
         <v>149</v>
       </c>
       <c r="AD4" t="n">
-        <v>0.0129567315706916</v>
+        <v>0.00520091438971038</v>
       </c>
       <c r="AE4" t="n">
         <v>1</v>
@@ -1014,7 +1008,7 @@
         <v>49</v>
       </c>
       <c r="AH4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="AI4" t="n">
         <v>0.0306840393066931</v>
@@ -1023,7 +1017,7 @@
         <v>46</v>
       </c>
       <c r="AK4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="AL4" t="n">
         <v>1</v>
@@ -1032,7 +1026,7 @@
         <v>1</v>
       </c>
       <c r="AN4" t="n">
-        <v>0.9</v>
+        <v>2.2421169701799</v>
       </c>
       <c r="AO4" t="n">
         <v>2</v>
@@ -1041,12 +1035,12 @@
         <v>0.5</v>
       </c>
       <c r="AQ4" t="n">
-        <v>0.0028</v>
+        <v>0.0069</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B5" t="n">
         <v>0.0371043179696165</v>
@@ -1121,10 +1115,10 @@
         <v>1940.05</v>
       </c>
       <c r="Z5" t="n">
-        <v>0.00597992354203657</v>
+        <v>0.0147237001953311</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.9</v>
+        <v>2.2421169701799</v>
       </c>
       <c r="AB5" t="n">
         <v>2.25243786750044</v>
@@ -1133,7 +1127,7 @@
         <v>69</v>
       </c>
       <c r="AD5" t="n">
-        <v>0.018303288432986</v>
+        <v>0.0073470562904511</v>
       </c>
       <c r="AE5" t="n">
         <v>1</v>
@@ -1145,7 +1139,7 @@
         <v>49</v>
       </c>
       <c r="AH5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="AI5" t="n">
         <v>0.0371349095748844</v>
@@ -1154,7 +1148,7 @@
         <v>46</v>
       </c>
       <c r="AK5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="AL5" t="n">
         <v>1</v>
@@ -1163,7 +1157,7 @@
         <v>1</v>
       </c>
       <c r="AN5" t="n">
-        <v>0.9</v>
+        <v>2.2421169701799</v>
       </c>
       <c r="AO5" t="n">
         <v>2</v>
@@ -1172,12 +1166,12 @@
         <v>0.5</v>
       </c>
       <c r="AQ5" t="n">
-        <v>0.006</v>
+        <v>0.015</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B6" t="n">
         <v>0.320860486165164</v>
@@ -1252,10 +1246,10 @@
         <v>2010</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.00671019667865075</v>
+        <v>0.0164996173784996</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.9</v>
+        <v>2.2421169701799</v>
       </c>
       <c r="AB6" t="n">
         <v>2.26655532256648</v>
@@ -1264,7 +1258,7 @@
         <v>62</v>
       </c>
       <c r="AD6" t="n">
-        <v>0.157292278615525</v>
+        <v>0.063138120194779</v>
       </c>
       <c r="AE6" t="n">
         <v>1</v>
@@ -1276,7 +1270,7 @@
         <v>49</v>
       </c>
       <c r="AH6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="AI6" t="n">
         <v>0.343466368449842</v>
@@ -1285,7 +1279,7 @@
         <v>46</v>
       </c>
       <c r="AK6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="AL6" t="n">
         <v>1</v>
@@ -1294,7 +1288,7 @@
         <v>1</v>
       </c>
       <c r="AN6" t="n">
-        <v>0.9</v>
+        <v>2.2421169701799</v>
       </c>
       <c r="AO6" t="n">
         <v>2</v>
@@ -1303,12 +1297,12 @@
         <v>0.5</v>
       </c>
       <c r="AQ6" t="n">
-        <v>0.0067</v>
+        <v>0.016</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B7" t="n">
         <v>0.358270947361978</v>
@@ -1383,10 +1377,10 @@
         <v>2055.53</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.00352057763911637</v>
+        <v>0.00871032854251671</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.9</v>
+        <v>2.2421169701799</v>
       </c>
       <c r="AB7" t="n">
         <v>2.26099319489918</v>
@@ -1395,7 +1389,7 @@
         <v>117</v>
       </c>
       <c r="AD7" t="n">
-        <v>0.176063701253178</v>
+        <v>0.0706730885298754</v>
       </c>
       <c r="AE7" t="n">
         <v>1</v>
@@ -1404,10 +1398,10 @@
         <v>1.07282929872356</v>
       </c>
       <c r="AG7" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="AH7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="AI7" t="n">
         <v>0.384363569211378</v>
@@ -1416,7 +1410,7 @@
         <v>46</v>
       </c>
       <c r="AK7" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="AL7" t="n">
         <v>0</v>
@@ -1425,7 +1419,7 @@
         <v>2</v>
       </c>
       <c r="AN7" t="n">
-        <v>0.9</v>
+        <v>2.2421169701799</v>
       </c>
       <c r="AO7" t="n">
         <v>2</v>
@@ -1434,12 +1428,12 @@
         <v>0.5</v>
       </c>
       <c r="AQ7" t="n">
-        <v>0.0035</v>
+        <v>0.0087</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B8" t="n">
         <v>0.0326813688912162</v>
@@ -1514,10 +1508,10 @@
         <v>1959.58</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.00248268162826229</v>
+        <v>0.00615500708319985</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.9</v>
+        <v>2.2421169701799</v>
       </c>
       <c r="AB8" t="n">
         <v>2.26751588714622</v>
@@ -1526,7 +1520,7 @@
         <v>166</v>
       </c>
       <c r="AD8" t="n">
-        <v>0.0160142790210182</v>
+        <v>0.00642823336632611</v>
       </c>
       <c r="AE8" t="n">
         <v>1</v>
@@ -1538,7 +1532,7 @@
         <v>49</v>
       </c>
       <c r="AH8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="AI8" t="n">
         <v>0.0327494414017846</v>
@@ -1547,7 +1541,7 @@
         <v>46</v>
       </c>
       <c r="AK8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="AL8" t="n">
         <v>1</v>
@@ -1556,7 +1550,7 @@
         <v>1</v>
       </c>
       <c r="AN8" t="n">
-        <v>0.9</v>
+        <v>2.2421169701799</v>
       </c>
       <c r="AO8" t="n">
         <v>2</v>
@@ -1565,12 +1559,12 @@
         <v>0.5</v>
       </c>
       <c r="AQ8" t="n">
-        <v>0.0025</v>
+        <v>0.0062</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B9" t="n">
         <v>0.0739757902704793</v>
@@ -1645,10 +1639,10 @@
         <v>1975.14</v>
       </c>
       <c r="Z9" t="n">
-        <v>0.00215149010227422</v>
+        <v>0.0053374072280561</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.9</v>
+        <v>2.2421169701799</v>
       </c>
       <c r="AB9" t="n">
         <v>2.27101733017835</v>
@@ -1657,7 +1651,7 @@
         <v>192</v>
       </c>
       <c r="AD9" t="n">
-        <v>0.0361931727382722</v>
+        <v>0.0145281695369495</v>
       </c>
       <c r="AE9" t="n">
         <v>1</v>
@@ -1669,7 +1663,7 @@
         <v>49</v>
       </c>
       <c r="AH9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="AI9" t="n">
         <v>0.0744366757599961</v>
@@ -1678,7 +1672,7 @@
         <v>46</v>
       </c>
       <c r="AK9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="AL9" t="n">
         <v>1</v>
@@ -1687,7 +1681,7 @@
         <v>1</v>
       </c>
       <c r="AN9" t="n">
-        <v>0.9</v>
+        <v>2.2421169701799</v>
       </c>
       <c r="AO9" t="n">
         <v>2</v>
@@ -1696,12 +1690,12 @@
         <v>0.5</v>
       </c>
       <c r="AQ9" t="n">
-        <v>0.0022</v>
+        <v>0.0053</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B10" t="n">
         <v>0.00933809045098793</v>
@@ -1776,10 +1770,10 @@
         <v>1948.32</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.00354180564350198</v>
+        <v>0.00876211089741444</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.9</v>
+        <v>2.2421169701799</v>
       </c>
       <c r="AB10" t="n">
         <v>2.24707891382181</v>
@@ -1788,7 +1782,7 @@
         <v>70</v>
       </c>
       <c r="AD10" t="n">
-        <v>0.00461739727645186</v>
+        <v>0.00185345260933164</v>
       </c>
       <c r="AE10" t="n">
         <v>1</v>
@@ -1800,7 +1794,7 @@
         <v>49</v>
       </c>
       <c r="AH10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="AI10" t="n">
         <v>0.00933095135088507</v>
@@ -1809,7 +1803,7 @@
         <v>46</v>
       </c>
       <c r="AK10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="AL10" t="n">
         <v>1</v>
@@ -1818,7 +1812,7 @@
         <v>1</v>
       </c>
       <c r="AN10" t="n">
-        <v>0.9</v>
+        <v>2.2421169701799</v>
       </c>
       <c r="AO10" t="n">
         <v>2</v>
@@ -1827,7 +1821,7 @@
         <v>0.5</v>
       </c>
       <c r="AQ10" t="n">
-        <v>0.0035</v>
+        <v>0.0088</v>
       </c>
     </row>
   </sheetData>

</xml_diff>